<commit_message>
validate uploaded spreadsheet filename
</commit_message>
<xml_diff>
--- a/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
+++ b/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sprior\source\repos\rsd-lsrp-validation-function\src\Tests\GovUK.Dfe.Lsrp.FileValidator.Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD30C2D8-77A0-400A-9C16-48FC0441162C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A2AF87-A835-42FF-96CB-AE3F71F99BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34440" yWindow="-4590" windowWidth="38640" windowHeight="21120" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
+    <workbookView xWindow="41040" yWindow="-1230" windowWidth="18675" windowHeight="10815" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="2" r:id="rId1"/>
@@ -49,7 +49,7 @@
     <t>The Local SEND Reform Plan</t>
   </si>
   <si>
-    <t>LA1</t>
+    <t>LA1 Local Authority 1</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Spreadsheet validation - filename (#17)
* validate uploaded filename

* improve validate uploaded filename tests

* enhance validate uploaded filename tests

* delete local authority provider and check LA code in message

* validate uploaded spreadsheet filename

* delete redundant financial quarter class

* Potential fix for pull request finding -  filename parsing

Co-authored-by: Copilot Autofix powered by AI <175728472+Copilot@users.noreply.github.com>

* add spreadsheet version to app settings

---------

Co-authored-by: PRIOR <Stephen.PRIOR@EDUCATION.GOV.UK>
Co-authored-by: Copilot Autofix powered by AI <175728472+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
+++ b/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sprior\source\repos\rsd-lsrp-validation-function\src\Tests\GovUK.Dfe.Lsrp.FileValidator.Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD30C2D8-77A0-400A-9C16-48FC0441162C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A2AF87-A835-42FF-96CB-AE3F71F99BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34440" yWindow="-4590" windowWidth="38640" windowHeight="21120" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
+    <workbookView xWindow="41040" yWindow="-1230" windowWidth="18675" windowHeight="10815" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="2" r:id="rId1"/>
@@ -49,7 +49,7 @@
     <t>The Local SEND Reform Plan</t>
   </si>
   <si>
-    <t>LA1</t>
+    <t>LA1 Local Authority 1</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
change validation rules to match latest spreadsheet template
</commit_message>
<xml_diff>
--- a/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
+++ b/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sprior\source\repos\rsd-lsrp-validation-function\src\Tests\GovUK.Dfe.Lsrp.FileValidator.Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A2AF87-A835-42FF-96CB-AE3F71F99BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCFA4D35-A369-48BB-925A-3DA52985A92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41040" yWindow="-1230" windowWidth="18675" windowHeight="10815" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
+    <workbookView xWindow="41040" yWindow="-1230" windowWidth="19230" windowHeight="11100" activeTab="1" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="2" r:id="rId1"/>
-    <sheet name="Guidance" sheetId="3" r:id="rId2"/>
-    <sheet name="Quarterly Returns" sheetId="1" r:id="rId3"/>
+    <sheet name="Quarterly Return Template" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,13 +42,13 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
-    <t>2026-27 Data</t>
-  </si>
-  <si>
     <t>The Local SEND Reform Plan</t>
   </si>
   <si>
     <t>LA1 Local Authority 1</t>
+  </si>
+  <si>
+    <t>2026-27 Quarterly Data</t>
   </si>
 </sst>
 </file>
@@ -426,7 +425,7 @@
   <sheetData>
     <row r="13" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -435,15 +434,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{527E68FE-6F8C-42C3-8377-B9605942753C}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{446C1C83-F5E7-4A1F-9701-4249491BCE9A}">
   <dimension ref="B4:B5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -453,12 +443,12 @@
   <sheetData>
     <row r="4" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
change validation rules to match latest spreadsheet template (#24)
Co-authored-by: PRIOR <Stephen.PRIOR@EDUCATION.GOV.UK>
</commit_message>
<xml_diff>
--- a/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
+++ b/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sprior\source\repos\rsd-lsrp-validation-function\src\Tests\GovUK.Dfe.Lsrp.FileValidator.Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A2AF87-A835-42FF-96CB-AE3F71F99BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCFA4D35-A369-48BB-925A-3DA52985A92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41040" yWindow="-1230" windowWidth="18675" windowHeight="10815" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
+    <workbookView xWindow="41040" yWindow="-1230" windowWidth="19230" windowHeight="11100" activeTab="1" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="2" r:id="rId1"/>
-    <sheet name="Guidance" sheetId="3" r:id="rId2"/>
-    <sheet name="Quarterly Returns" sheetId="1" r:id="rId3"/>
+    <sheet name="Quarterly Return Template" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,13 +42,13 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
-    <t>2026-27 Data</t>
-  </si>
-  <si>
     <t>The Local SEND Reform Plan</t>
   </si>
   <si>
     <t>LA1 Local Authority 1</t>
+  </si>
+  <si>
+    <t>2026-27 Quarterly Data</t>
   </si>
 </sst>
 </file>
@@ -426,7 +425,7 @@
   <sheetData>
     <row r="13" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -435,15 +434,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{527E68FE-6F8C-42C3-8377-B9605942753C}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{446C1C83-F5E7-4A1F-9701-4249491BCE9A}">
   <dimension ref="B4:B5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -453,12 +443,12 @@
   <sheetData>
     <row r="4" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>